<commit_message>
PM spreadsheet: S17–S21 and the Oct 2026 plan (M1–M4 done)
Dashboard figures and velocity rows, session diary S17–S21, decision
records 16–22, backlog items done (#39 cloud sync, #40 export/import,
pricing), a new milestone table for the Oct 2026 plan (old M7 marked as
replaced), feature registry 56–70. History rows left unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KlimaChallenge_PM_v5.xlsx
+++ b/docs/KlimaChallenge_PM_v5.xlsx
@@ -2308,7 +2308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="238" min="1" max="1"/>
@@ -2342,7 +2342,7 @@
     <row r="2" ht="18" customHeight="1" s="239">
       <c r="A2" s="242" t="inlineStr">
         <is>
-          <t>Session 16 Complete  ·  2026-03-16  ·  React Native / Expo SDK 54  ·  Supabase  ·  TypeScript</t>
+          <t>Session 21 Complete  ·  2026-10-21  ·  Prototype phase (Oct 2026 plan): M1–M4 done  ·  Expo SDK 54  ·  Supabase  ·  TypeScript</t>
         </is>
       </c>
       <c r="B2" s="241" t="n"/>
@@ -2400,19 +2400,19 @@
     <row r="6" ht="36" customHeight="1" s="239">
       <c r="A6" s="250" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B6" s="251" t="n"/>
       <c r="C6" s="252" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>70</t>
         </is>
       </c>
       <c r="D6" s="251" t="n"/>
       <c r="E6" s="253" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F6" s="251" t="n"/>
@@ -2424,7 +2424,7 @@
       <c r="H6" s="251" t="n"/>
       <c r="I6" s="255" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J6" s="251" t="n"/>
@@ -2432,7 +2432,7 @@
     <row r="7" ht="15.75" customHeight="1" s="239">
       <c r="A7" s="256" t="inlineStr">
         <is>
-          <t>prev sessions: 15 / 44 / 11 / 0 / 5   · Open Backlog = open feature/bug items; Pre-Prod Blockers = separate infra items not counted above</t>
+          <t>prev (S16): 16 / 46 / 10 / 0 / 5   · Features now counted from the Feature Registry (55 at S16, 70 at S21) · Backlog figures from the Backlog sheet; since Oct 2026 the live task list is ROADMAP.md</t>
         </is>
       </c>
       <c r="B7" s="241" t="n"/>
@@ -2703,7 +2703,7 @@
       <c r="E17" s="263" t="n"/>
       <c r="F17" s="264" t="inlineStr">
         <is>
-          <t>🔄 In Progress  (30%)</t>
+          <t>⏸ Replaced (Oct 2026 plan)</t>
         </is>
       </c>
       <c r="G17" s="263" t="n"/>
@@ -2715,7 +2715,7 @@
       <c r="I17" s="263" t="n"/>
       <c r="J17" s="265" t="inlineStr">
         <is>
-          <t>Bugs #36/#37 ✓ fixed S13. Remaining: pricing API (PP2), email confirm (PP1), onboarding rework #44, images (PP3), App Store assets (PP4), EAS build (PP5)</t>
+          <t>Not finished as planned; work resumed in Oct 2026 under a new plan (PROTOTYPE PHASE below). Pricing (PP2) solved by the ÖBB fare model in S19.</t>
         </is>
       </c>
     </row>
@@ -3300,8 +3300,499 @@
         </is>
       </c>
     </row>
+    <row r="38" ht="18" customHeight="1" s="239">
+      <c r="A38" s="266" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="B38" s="267" t="inlineStr">
+        <is>
+          <t>Apr 15</t>
+        </is>
+      </c>
+      <c r="C38" s="268" t="inlineStr">
+        <is>
+          <t>Trello board with full project history + sync tooling</t>
+        </is>
+      </c>
+      <c r="D38" s="280" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E38" s="270" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="F38" s="271" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="281" t="inlineStr">
+        <is>
+          <t>░░░░░░░░░░</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="239">
+      <c r="A39" s="273" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="B39" s="274" t="inlineStr">
+        <is>
+          <t>Apr 20</t>
+        </is>
+      </c>
+      <c r="C39" s="275" t="inlineStr">
+        <is>
+          <t>Trip export/import (JSON), UUID trip IDs, cloud sync prep</t>
+        </is>
+      </c>
+      <c r="D39" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="277" t="inlineStr">
+        <is>
+          <t>Feature / Data</t>
+        </is>
+      </c>
+      <c r="F39" s="278" t="n">
+        <v>58</v>
+      </c>
+      <c r="G39" s="279" t="inlineStr">
+        <is>
+          <t>█░░░░░░░░░</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="239">
+      <c r="A40" s="266" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="B40" s="267" t="inlineStr">
+        <is>
+          <t>Oct 20</t>
+        </is>
+      </c>
+      <c r="C40" s="268" t="inlineStr">
+        <is>
+          <t>Restart: cleanup, ÖBB Open Data trip entry, anonymous sign-in, shared store (M1–M3)</t>
+        </is>
+      </c>
+      <c r="D40" s="280" t="n">
+        <v>9</v>
+      </c>
+      <c r="E40" s="270" t="inlineStr">
+        <is>
+          <t>Infra / Data / Feature</t>
+        </is>
+      </c>
+      <c r="F40" s="271" t="n">
+        <v>67</v>
+      </c>
+      <c r="G40" s="281" t="inlineStr">
+        <is>
+          <t>██████████</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="239">
+      <c r="A41" s="273" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="B41" s="274" t="inlineStr">
+        <is>
+          <t>Oct 21</t>
+        </is>
+      </c>
+      <c r="C41" s="275" t="inlineStr">
+        <is>
+          <t>Recap; all open study and design questions answered; project log</t>
+        </is>
+      </c>
+      <c r="D41" s="276" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E41" s="277" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="F41" s="278" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="279" t="inlineStr">
+        <is>
+          <t>░░░░░░░░░░</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="239">
+      <c r="A42" s="266" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="B42" s="267" t="inlineStr">
+        <is>
+          <t>Oct 21</t>
+        </is>
+      </c>
+      <c r="C42" s="268" t="inlineStr">
+        <is>
+          <t>Cloud backup (M4): sync, restore, merge question, study export; −XP toast</t>
+        </is>
+      </c>
+      <c r="D42" s="280" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" s="270" t="inlineStr">
+        <is>
+          <t>Data / Feature</t>
+        </is>
+      </c>
+      <c r="F42" s="271" t="n">
+        <v>72</v>
+      </c>
+      <c r="G42" s="281" t="inlineStr">
+        <is>
+          <t>██████░░░░</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="7.5" customHeight="1" s="239">
+      <c r="A43" s="243" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="239">
+      <c r="A44" s="244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PROTOTYPE PHASE — MILESTONES  (plan of 20 Oct 2026; details in ROADMAP.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1" s="239">
+      <c r="A45" s="257" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B45" s="257" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="C45" s="257" t="n"/>
+      <c r="D45" s="257" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="E45" s="257" t="n"/>
+      <c r="F45" s="257" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G45" s="257" t="n"/>
+      <c r="H45" s="257" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="I45" s="257" t="n"/>
+      <c r="J45" s="257" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="19.5" customHeight="1" s="239">
+      <c r="A46" s="258" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="B46" s="259" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="D46" s="259" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F46" s="260" t="inlineStr">
+        <is>
+          <t>✅ Complete (100%)</t>
+        </is>
+      </c>
+      <c r="H46" s="259" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J46" s="259" t="inlineStr">
+        <is>
+          <t>Repo cleanup, SDK 54 deps, ESLint + Prettier, tsc 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="19.5" customHeight="1" s="239">
+      <c r="A47" s="258" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B47" s="259" t="inlineStr">
+        <is>
+          <t>Trip entry + fixes</t>
+        </is>
+      </c>
+      <c r="D47" s="259" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F47" s="260" t="inlineStr">
+        <is>
+          <t>✅ Complete (100%)</t>
+        </is>
+      </c>
+      <c r="H47" s="259" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J47" s="259" t="inlineStr">
+        <is>
+          <t>ÖBB Open Data stations, distances, fares; anonymous sign-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="19.5" customHeight="1" s="239">
+      <c r="A48" s="258" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B48" s="259" t="inlineStr">
+        <is>
+          <t>Data core</t>
+        </is>
+      </c>
+      <c r="D48" s="259" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F48" s="260" t="inlineStr">
+        <is>
+          <t>✅ Complete (100%)</t>
+        </is>
+      </c>
+      <c r="H48" s="259" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J48" s="259" t="inlineStr">
+        <is>
+          <t>Shared store, derived XP, ticket periods; 76 tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="19.5" customHeight="1" s="239">
+      <c r="A49" s="258" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B49" s="259" t="inlineStr">
+        <is>
+          <t>Cloud backup</t>
+        </is>
+      </c>
+      <c r="D49" s="259" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="F49" s="260" t="inlineStr">
+        <is>
+          <t>✅ Complete (100%)</t>
+        </is>
+      </c>
+      <c r="H49" s="259" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J49" s="259" t="inlineStr">
+        <is>
+          <t>Done 21 Oct: backup + restore, merge question, study export; 106 tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="19.5" customHeight="1" s="239">
+      <c r="A50" s="261" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B50" s="262" t="inlineStr">
+        <is>
+          <t>Polish + insights (+ M5b gamification)</t>
+        </is>
+      </c>
+      <c r="C50" s="263" t="n"/>
+      <c r="D50" s="262" t="inlineStr">
+        <is>
+          <t>2026-12-18</t>
+        </is>
+      </c>
+      <c r="E50" s="263" t="n"/>
+      <c r="F50" s="264" t="inlineStr">
+        <is>
+          <t>⬜ Next</t>
+        </is>
+      </c>
+      <c r="G50" s="263" t="n"/>
+      <c r="H50" s="264" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I50" s="263" t="n"/>
+      <c r="J50" s="265" t="inlineStr">
+        <is>
+          <t>German + English, onboarding rework, weekly goal ladder</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="19.5" customHeight="1" s="239">
+      <c r="A51" s="261" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B51" s="262" t="inlineStr">
+        <is>
+          <t>Study-ready</t>
+        </is>
+      </c>
+      <c r="C51" s="263" t="n"/>
+      <c r="D51" s="262" t="inlineStr">
+        <is>
+          <t>2027-01-10</t>
+        </is>
+      </c>
+      <c r="E51" s="263" t="n"/>
+      <c r="F51" s="264" t="inlineStr">
+        <is>
+          <t>⬜ Planned</t>
+        </is>
+      </c>
+      <c r="G51" s="263" t="n"/>
+      <c r="H51" s="264" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I51" s="263" t="n"/>
+      <c r="J51" s="265" t="inlineStr">
+        <is>
+          <t>Consent + study code, APK / TestFlight, weekly export</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="19.5" customHeight="1" s="239">
+      <c r="A52" s="261" t="inlineStr">
+        <is>
+          <t>Pilot</t>
+        </is>
+      </c>
+      <c r="B52" s="262" t="inlineStr">
+        <is>
+          <t>Pilot test (5–8 people)</t>
+        </is>
+      </c>
+      <c r="C52" s="263" t="n"/>
+      <c r="D52" s="262" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="E52" s="263" t="n"/>
+      <c r="F52" s="264" t="inlineStr">
+        <is>
+          <t>⬜ Planned</t>
+        </is>
+      </c>
+      <c r="G52" s="263" t="n"/>
+      <c r="H52" s="264" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I52" s="263" t="n"/>
+      <c r="J52" s="265" t="inlineStr">
+        <is>
+          <t>30 Nov – 13 Dec, Android only</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="19.5" customHeight="1" s="239">
+      <c r="A53" s="261" t="inlineStr">
+        <is>
+          <t>Study</t>
+        </is>
+      </c>
+      <c r="B53" s="262" t="inlineStr">
+        <is>
+          <t>User study (6 weeks)</t>
+        </is>
+      </c>
+      <c r="C53" s="263" t="n"/>
+      <c r="D53" s="262" t="inlineStr">
+        <is>
+          <t>2027-02-21</t>
+        </is>
+      </c>
+      <c r="E53" s="263" t="n"/>
+      <c r="F53" s="264" t="inlineStr">
+        <is>
+          <t>⬜ Planned</t>
+        </is>
+      </c>
+      <c r="G53" s="263" t="n"/>
+      <c r="H53" s="264" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I53" s="263" t="n"/>
+      <c r="J53" s="265" t="inlineStr">
+        <is>
+          <t>11 Jan – 21 Feb; submission 31 Mar 2027</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="20">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="C6:D6"/>
@@ -3320,6 +3811,8 @@
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A43:J43"/>
+    <mergeCell ref="A44:J44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3334,7 +3827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="238" min="1" max="1"/>
@@ -4422,8 +4915,312 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="239">
-      <c r="A21" s="328" t="inlineStr">
+    <row r="21" ht="120" customHeight="1" s="239">
+      <c r="A21" s="322" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="B21" s="323" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="C21" s="324" t="inlineStr">
+        <is>
+          <t>Trello board + sync tooling</t>
+        </is>
+      </c>
+      <c r="D21" s="305" t="inlineStr">
+        <is>
+          <t>Created a Trello board via API with the full project history (70 cards, effort labels); trello_sync.js CLI for ongoing sync. Backlog: #40 export/import expanded, new #52 trip generator wizard.</t>
+        </is>
+      </c>
+      <c r="E21" s="306" t="inlineStr">
+        <is>
+          <t>Visual project tracking alongside the spreadsheet.</t>
+        </is>
+      </c>
+      <c r="F21" s="307" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="308" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="309" t="inlineStr">
+        <is>
+          <t>The Trello token ended up committed in .claude/settings.local.json (expired May 2026; the file was untracked in S19).</t>
+        </is>
+      </c>
+      <c r="I21" s="325" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" s="326" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K21" s="327" t="inlineStr">
+        <is>
+          <t>Development Process / Tooling</t>
+        </is>
+      </c>
+      <c r="L21" s="313" t="inlineStr">
+        <is>
+          <t>Retired in S19: one roadmap file in the repo plus a project log doc proved easier to keep current than several trackers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="120" customHeight="1" s="239">
+      <c r="A22" s="322" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="B22" s="323" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="C22" s="324" t="inlineStr">
+        <is>
+          <t>Trip export/import + cloud sync preparation</t>
+        </is>
+      </c>
+      <c r="D22" s="305" t="inlineStr">
+        <is>
+          <t>services/tripExport.ts: export trips as JSON via the share sheet, import via document picker (merge by trip ID, duplicates skipped); Data section in the profile. initialTrips dead code removed; trip IDs switched to UUIDs (generateTripId). Cloud sync plan written (phases 0–4).</t>
+        </is>
+      </c>
+      <c r="E22" s="306" t="inlineStr">
+        <is>
+          <t>A manual backup before cloud sync existed. UUIDs are the prerequisite for merging data from several phones without duplicates.</t>
+        </is>
+      </c>
+      <c r="F22" s="307" t="inlineStr">
+        <is>
+          <t>crypto.randomUUID() was assumed to exist on Hermes; it does not (trip creation crashed, fixed in S19 with a fallback).</t>
+        </is>
+      </c>
+      <c r="G22" s="308" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="309" t="inlineStr">
+        <is>
+          <t>Never assume a web API exists on Hermes: test on the device.</t>
+        </is>
+      </c>
+      <c r="I22" s="325" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="326" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K22" s="327" t="inlineStr">
+        <is>
+          <t>Data Architecture</t>
+        </is>
+      </c>
+      <c r="L22" s="313" t="inlineStr">
+        <is>
+          <t>UUID trip IDs paid off in M4: adding a phone's anonymous trips to an account needs no duplicate handling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="120" customHeight="1" s="239">
+      <c r="A23" s="322" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="B23" s="323" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C23" s="324" t="inlineStr">
+        <is>
+          <t>Restart after six months: review + M1–M3</t>
+        </is>
+      </c>
+      <c r="D23" s="305" t="inlineStr">
+        <is>
+          <t>Read-only review; PC set up again (Node, adb, dev build on Xiaomi 11T Pro). M1: LF line endings, deps aligned with SDK 54, ESLint + Prettier, tsc 0. M2: anonymous sign-in + optional account on the same user ID; ÖBB Open Data pipeline (1,117 stations, GTFS rail network with Dijkstra, fare model fitted to Relationspreise); new Quick Add flow; Check price at ÖBB. M3: shared AppData store, XP derived from trips + reward-claim log, ticket periods, net savings; 76 tests.</t>
+        </is>
+      </c>
+      <c r="E23" s="306" t="inlineStr">
+        <is>
+          <t>Thesis due end of March 2027 with a user study in Jan–Feb: the app had to become reliable and measurable first. The ÖBB proxy was dead and the stored XP counter drifted from the data.</t>
+        </is>
+      </c>
+      <c r="F23" s="307" t="inlineStr">
+        <is>
+          <t>oebb.macistry.com returned 503 (service suspended): connection search and distances stopped working. Trip creation crashed (no global crypto on Hermes). Verbund fares are higher than the ÖBB standard fare (e.g. €10.50 vs €8.60 Villach–Klagenfurt).</t>
+        </is>
+      </c>
+      <c r="G23" s="308" t="inlineStr">
+        <is>
+          <t>Another unofficial proxy or scraping ÖBB prices (bot check) rejected; patching the stored XP counter rejected in favour of deriving XP.</t>
+        </is>
+      </c>
+      <c r="H23" s="309" t="inlineStr">
+        <is>
+          <t>Run as a development build, not Expo Go. Screenshots via adb exec-out from Bash; taps are blocked by Xiaomi security. Check the Test Suites line, not only Tests.</t>
+        </is>
+      </c>
+      <c r="I23" s="325" t="n">
+        <v>9</v>
+      </c>
+      <c r="J23" s="326" t="inlineStr">
+        <is>
+          <t>~10h</t>
+        </is>
+      </c>
+      <c r="K23" s="327" t="inlineStr">
+        <is>
+          <t>Data Architecture / Data Sources / Gamification Design</t>
+        </is>
+      </c>
+      <c r="L23" s="313" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="120" customHeight="1" s="239">
+      <c r="A24" s="322" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="B24" s="323" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C24" s="324" t="inlineStr">
+        <is>
+          <t>Recap + study and design decisions</t>
+        </is>
+      </c>
+      <c r="D24" s="305" t="inlineStr">
+        <is>
+          <t>Status and recap doc; all 14 open questions answered (participants, hypothetical tickets, consent with study code, one trip = whole journey, reminders, gamification set, weekly goal ladder, reward revocation, community total, Supabase plan, documentation). Project Log doc created; branch pushed.</t>
+        </is>
+      </c>
+      <c r="E24" s="306" t="inlineStr">
+        <is>
+          <t>The study design decides what the app must record, so it had to be settled before M4–M6.</t>
+        </is>
+      </c>
+      <c r="F24" s="307" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="308" t="inlineStr">
+        <is>
+          <t>Daily streak replaced by a weekly goal ladder (daily streaks punish weekends and part-timers). Leaderboards rejected (privacy, can discourage).</t>
+        </is>
+      </c>
+      <c r="H24" s="309" t="inlineStr">
+        <is>
+          <t>Decisions recorded in ROADMAP.md and the Project Log.</t>
+        </is>
+      </c>
+      <c r="I24" s="325" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" s="326" t="inlineStr">
+        <is>
+          <t>~1h</t>
+        </is>
+      </c>
+      <c r="K24" s="327" t="inlineStr">
+        <is>
+          <t>Study Design / Gamification Theory</t>
+        </is>
+      </c>
+      <c r="L24" s="313" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="120" customHeight="1" s="239">
+      <c r="A25" s="322" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="B25" s="323" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C25" s="324" t="inlineStr">
+        <is>
+          <t>M4 cloud backup</t>
+        </is>
+      </c>
+      <c r="D25" s="305" t="inlineStr">
+        <is>
+          <t>Supabase migration: trips, reward_claims, profiles with row-level security; server-set synced_at; last-writer-wins trigger; study schema with views without station names. utils/syncLogic.ts (pure, tested), services/cloudSync.ts, store integration: outbox, retries, restore on login, merge question, logout that syncs first. Backup status icon; red −XP toast. 106 tests incl. store tests against an in-memory Supabase fake. Tested on the phone.</t>
+        </is>
+      </c>
+      <c r="E25" s="306" t="inlineStr">
+        <is>
+          <t>An account without restore felt broken, and the same tables provide the study data, replacing the one-way upload planned earlier.</t>
+        </is>
+      </c>
+      <c r="F25" s="307" t="inlineStr">
+        <is>
+          <t>No service key, so the user ran the SQL in the dashboard. Repeated sync rounds could show the merge question twice (fixed). Merged anonymous trips stay in the cloud under an anonymous user nobody can reach.</t>
+        </is>
+      </c>
+      <c r="G25" s="308" t="inlineStr">
+        <is>
+          <t>Real-time subscriptions (not needed for one person on one or two phones); a server function that moves anonymous rows to the account (anyone knowing an ID could take the data).</t>
+        </is>
+      </c>
+      <c r="H25" s="309" t="inlineStr">
+        <is>
+          <t>Trip primary key is (user_id, id), so the same trip can exist once per user. The study views leave out anonymous users whose trips were merged, so nothing is counted twice.</t>
+        </is>
+      </c>
+      <c r="I25" s="325" t="n">
+        <v>5</v>
+      </c>
+      <c r="J25" s="326" t="inlineStr">
+        <is>
+          <t>~2h</t>
+        </is>
+      </c>
+      <c r="K25" s="327" t="inlineStr">
+        <is>
+          <t>Data Architecture / Privacy / Research Data</t>
+        </is>
+      </c>
+      <c r="L25" s="313" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1" s="239">
+      <c r="A26" s="328" t="inlineStr">
         <is>
           <t>Column colour guide:  E (green) = Why / rationale  ·  F (red) = Problems  ·  H (blue) = Standing decisions  ·  L (purple) = Retrospective reflection</t>
         </is>
@@ -4448,7 +5245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="238" min="1" max="1"/>
@@ -5146,6 +5943,286 @@
       <c r="H19" s="363" t="inlineStr">
         <is>
           <t>S16</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="100" customHeight="1" s="239">
+      <c r="A20" s="349" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="344" t="inlineStr">
+        <is>
+          <t>Sign-in model</t>
+        </is>
+      </c>
+      <c r="C20" s="345" t="inlineStr">
+        <is>
+          <t>Study participants should start without hurdles, but data must survive a phone change.</t>
+        </is>
+      </c>
+      <c r="D20" s="346" t="inlineStr">
+        <is>
+          <t>Email account required · anonymous only · anonymous by default with an optional account</t>
+        </is>
+      </c>
+      <c r="E20" s="347" t="inlineStr">
+        <is>
+          <t>Anonymous Supabase sign-in on first launch; an optional account upgrades the same user ID (updateUser), so no data has to be moved.</t>
+        </is>
+      </c>
+      <c r="F20" s="345" t="inlineStr">
+        <is>
+          <t>Low hurdle, little personal data, restore possible.</t>
+        </is>
+      </c>
+      <c r="G20" s="348" t="inlineStr">
+        <is>
+          <t>Low: requiring accounts later only changes onboarding.</t>
+        </is>
+      </c>
+      <c r="H20" s="349" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="100" customHeight="1" s="239">
+      <c r="A21" s="363" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="358" t="inlineStr">
+        <is>
+          <t>Station, distance and price data</t>
+        </is>
+      </c>
+      <c r="C21" s="359" t="inlineStr">
+        <is>
+          <t>The ÖBB proxy (macistry) was suspended; connection search and distances failed.</t>
+        </is>
+      </c>
+      <c r="D21" s="360" t="inlineStr">
+        <is>
+          <t>Another unofficial proxy · scraping the ÖBB shop · bundled ÖBB Open Data (GTFS, Relationspreise)</t>
+        </is>
+      </c>
+      <c r="E21" s="361" t="inlineStr">
+        <is>
+          <t>Bundled open data: 1,117 stations, rail distances via Dijkstra on the GTFS network, fare model fitted to Relationspreise (median deviation 4.9%); price editable and remembered per route.</t>
+        </is>
+      </c>
+      <c r="F21" s="359" t="inlineStr">
+        <is>
+          <t>Works offline, stable, licensed (CC BY 4.0), reproducible for the thesis.</t>
+        </is>
+      </c>
+      <c r="G21" s="362" t="inlineStr">
+        <is>
+          <t>Medium: the data must be regenerated for 2027 (pipeline in scripts/data).</t>
+        </is>
+      </c>
+      <c r="H21" s="363" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="100" customHeight="1" s="239">
+      <c r="A22" s="349" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="344" t="inlineStr">
+        <is>
+          <t>XP storage</t>
+        </is>
+      </c>
+      <c r="C22" s="345" t="inlineStr">
+        <is>
+          <t>The stored XP counter drifted from the trips (edits, deletes, imports).</t>
+        </is>
+      </c>
+      <c r="D22" s="346" t="inlineStr">
+        <is>
+          <t>Keep the counter and patch every code path · derive XP from the data</t>
+        </is>
+      </c>
+      <c r="E22" s="347" t="inlineStr">
+        <is>
+          <t>XP = trip XP + XP of claimed rewards in a timestamped claim log; nothing derived is stored. One-time migration of the old layout.</t>
+        </is>
+      </c>
+      <c r="F22" s="345" t="inlineStr">
+        <is>
+          <t>Always consistent; claims become study data.</t>
+        </is>
+      </c>
+      <c r="G22" s="348" t="inlineStr">
+        <is>
+          <t>Low.</t>
+        </is>
+      </c>
+      <c r="H22" s="349" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="100" customHeight="1" s="239">
+      <c r="A23" s="363" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="358" t="inlineStr">
+        <is>
+          <t>Cloud backup design</t>
+        </is>
+      </c>
+      <c r="C23" s="359" t="inlineStr">
+        <is>
+          <t>Trips must survive a phone change and feed the study export; the app must keep working offline.</t>
+        </is>
+      </c>
+      <c r="D23" s="360" t="inlineStr">
+        <is>
+          <t>One-way study upload · full real-time sync · local-first outbox with background upload and incremental download</t>
+        </is>
+      </c>
+      <c r="E23" s="361" t="inlineStr">
+        <is>
+          <t>Local-first: every change is saved on the phone and queued; the background sync uploads it and downloads rows changed since the last server time (synced_at). The later edit wins (updated_at, server trigger); deletions set deleted_at.</t>
+        </is>
+      </c>
+      <c r="F23" s="359" t="inlineStr">
+        <is>
+          <t>Offline-safe, no data loss, simple enough for one person on one or two phones.</t>
+        </is>
+      </c>
+      <c r="G23" s="362" t="inlineStr">
+        <is>
+          <t>Medium: real-time sync would replace the download loop; the tables stay.</t>
+        </is>
+      </c>
+      <c r="H23" s="363" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="100" customHeight="1" s="239">
+      <c r="A24" s="349" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="344" t="inlineStr">
+        <is>
+          <t>Anonymous trips when logging in to an existing account</t>
+        </is>
+      </c>
+      <c r="C24" s="345" t="inlineStr">
+        <is>
+          <t>A phone used without an account holds trips under an anonymous user ID; the account has its own.</t>
+        </is>
+      </c>
+      <c r="D24" s="346" t="inlineStr">
+        <is>
+          <t>Always merge · always discard · ask</t>
+        </is>
+      </c>
+      <c r="E24" s="347" t="inlineStr">
+        <is>
+          <t>Ask: "Add the N trips from this phone to your account?" Yes merges (UUID trip IDs, no duplicates), No keeps only the account's data.</t>
+        </is>
+      </c>
+      <c r="F24" s="345" t="inlineStr">
+        <is>
+          <t>The user stays in control of their data.</t>
+        </is>
+      </c>
+      <c r="G24" s="348" t="inlineStr">
+        <is>
+          <t>Low.</t>
+        </is>
+      </c>
+      <c r="H24" s="349" t="inlineStr">
+        <is>
+          <t>S19 / S21</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="100" customHeight="1" s="239">
+      <c r="A25" s="363" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="358" t="inlineStr">
+        <is>
+          <t>Study data export</t>
+        </is>
+      </c>
+      <c r="C25" s="359" t="inlineStr">
+        <is>
+          <t>The study needs usage data without identifying details; merged trips exist twice in the cloud.</t>
+        </is>
+      </c>
+      <c r="D25" s="360" t="inlineStr">
+        <is>
+          <t>Export script with the service key · views in the API schema · views in a separate schema</t>
+        </is>
+      </c>
+      <c r="E25" s="361" t="inlineStr">
+        <is>
+          <t>Views study.trips, study.rewards and study.tickets in a schema the app's API does not expose; no station names or free text; anonymous users whose trips were merged are left out.</t>
+        </is>
+      </c>
+      <c r="F25" s="359" t="inlineStr">
+        <is>
+          <t>Privacy, no double counting, only the researcher (dashboard) can read it.</t>
+        </is>
+      </c>
+      <c r="G25" s="362" t="inlineStr">
+        <is>
+          <t>Low.</t>
+        </is>
+      </c>
+      <c r="H25" s="363" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="100" customHeight="1" s="239">
+      <c r="A26" s="349" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="344" t="inlineStr">
+        <is>
+          <t>Streak mechanic</t>
+        </is>
+      </c>
+      <c r="C26" s="345" t="inlineStr">
+        <is>
+          <t>A daily streak punishes weekends and part-time commuters.</t>
+        </is>
+      </c>
+      <c r="D26" s="346" t="inlineStr">
+        <is>
+          <t>Keep the daily streak · weekly goal ladder</t>
+        </is>
+      </c>
+      <c r="E26" s="347" t="inlineStr">
+        <is>
+          <t>Weekly goal ladder: active days per week, +1 suggested after each met week, cap 5, one pause per month; streak = consecutive weeks with the goal met.</t>
+        </is>
+      </c>
+      <c r="F26" s="345" t="inlineStr">
+        <is>
+          <t>Achievable but rising goals; fewer incentives for fake trips.</t>
+        </is>
+      </c>
+      <c r="G26" s="348" t="inlineStr">
+        <is>
+          <t>Low (not built yet, M5b).</t>
+        </is>
+      </c>
+      <c r="H26" s="349" t="inlineStr">
+        <is>
+          <t>S20</t>
         </is>
       </c>
     </row>
@@ -5189,7 +6266,7 @@
     <row r="2" ht="18" customHeight="1" s="239">
       <c r="A2" s="288" t="inlineStr">
         <is>
-          <t>Priority-ordered work queue — open items first, pre-prod checklist second, completed archive below.</t>
+          <t>Priority-ordered work queue — open items first, pre-prod checklist second, completed archive below. · Since Oct 2026 the live task list is ROADMAP.md in the repository.</t>
         </is>
       </c>
     </row>
@@ -5392,143 +6469,143 @@
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" s="239">
-      <c r="A9" s="370" t="inlineStr">
+      <c r="A9" s="365" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="B9" s="370" t="inlineStr">
+      <c r="B9" s="366" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="C9" s="370" t="inlineStr">
+      <c r="C9" s="365" t="inlineStr">
         <is>
           <t>Cloud sync for trips (Supabase)</t>
         </is>
       </c>
-      <c r="D9" s="370" t="inlineStr">
+      <c r="D9" s="366" t="inlineStr">
         <is>
           <t>Trips stored AsyncStorage-only — new device login starts from scratch. No cross-device continuity.</t>
         </is>
       </c>
-      <c r="E9" s="371" t="inlineStr">
+      <c r="E9" s="366" t="inlineStr">
         <is>
           <t>🟠 High</t>
         </is>
       </c>
-      <c r="F9" s="370" t="inlineStr">
+      <c r="F9" s="366" t="inlineStr">
         <is>
           <t>L (1-2d)</t>
         </is>
       </c>
-      <c r="G9" s="370" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H9" s="370" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="I9" s="370" t="inlineStr">
-        <is>
-          <t>Requires Supabase trips table schema, upsert on save, fetch on login, conflict resolution</t>
+      <c r="G9" s="367" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H9" s="368" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="I9" s="369" t="inlineStr">
+        <is>
+          <t>Built in M4: Supabase tables with row-level security, local-first sync, restore on login, merge question (see ROADMAP.md).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1" s="239">
-      <c r="A10" s="372" t="inlineStr">
+      <c r="A10" s="365" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="B10" s="372" t="inlineStr">
+      <c r="B10" s="366" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="C10" s="372" t="inlineStr">
+      <c r="C10" s="365" t="inlineStr">
         <is>
           <t>Trip export / CSV download</t>
         </is>
       </c>
-      <c r="D10" s="372" t="inlineStr">
+      <c r="D10" s="366" t="inlineStr">
         <is>
           <t>Allow users to export all trips as CSV for tax/Jobticket employer reimbursement purposes.</t>
         </is>
       </c>
-      <c r="E10" s="373" t="inlineStr">
+      <c r="E10" s="366" t="inlineStr">
         <is>
           <t>🔵 Low</t>
         </is>
       </c>
-      <c r="F10" s="372" t="inlineStr">
+      <c r="F10" s="366" t="inlineStr">
         <is>
           <t>S (2-4h)</t>
         </is>
       </c>
-      <c r="G10" s="372" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H10" s="372" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="I10" s="372" t="inlineStr">
-        <is>
-          <t>expo-sharing + expo-file-system to write and share CSV file</t>
+      <c r="G10" s="367" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H10" s="368" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="I10" s="369" t="inlineStr">
+        <is>
+          <t>Built as JSON export/import (services/tripExport.ts); a CSV export was not built.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1" s="239">
-      <c r="A11" s="370" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B11" s="370" t="inlineStr">
+      <c r="A11" s="365" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B11" s="366" t="inlineStr">
         <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="C11" s="370" t="inlineStr">
+      <c r="C11" s="365" t="inlineStr">
         <is>
           <t>Pricing API investigation — pre-release priority</t>
         </is>
       </c>
-      <c r="D11" s="370" t="inlineStr">
+      <c r="D11" s="366" t="inlineStr">
         <is>
           <t>macistry HAFAS proxy returns no ticket prices. Candidates: ÖBB Scotty API, VAO, scraping ÖBB.at. Should be resolved before any public release — accurate pricing is core to the value proposition.</t>
         </is>
       </c>
-      <c r="E11" s="371" t="inlineStr">
+      <c r="E11" s="366" t="inlineStr">
         <is>
           <t>🟠 High</t>
         </is>
       </c>
-      <c r="F11" s="370" t="inlineStr">
+      <c r="F11" s="366" t="inlineStr">
         <is>
           <t>M (4-6h)</t>
         </is>
       </c>
-      <c r="G11" s="370" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H11" s="370" t="inlineStr">
-        <is>
-          <t>Pre-release</t>
-        </is>
-      </c>
-      <c r="I11" s="370" t="inlineStr">
-        <is>
-          <t>Elevated to High priority — this directly affects the accuracy of the app's core feature. See ADR #9.</t>
+      <c r="G11" s="367" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H11" s="368" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="I11" s="369" t="inlineStr">
+        <is>
+          <t>Solved with bundled ÖBB Open Data: fare model fitted to Relationspreise (median deviation 4.9%), editable, remembered per route.</t>
         </is>
       </c>
     </row>
@@ -6199,49 +7276,49 @@
       </c>
     </row>
     <row r="28" ht="25.5" customHeight="1" s="239">
-      <c r="A28" s="275" t="inlineStr">
+      <c r="A28" s="365" t="inlineStr">
         <is>
           <t>PP2</t>
         </is>
       </c>
-      <c r="B28" s="275" t="inlineStr">
+      <c r="B28" s="366" t="inlineStr">
         <is>
           <t>Pre-Prod</t>
         </is>
       </c>
-      <c r="C28" s="275" t="inlineStr">
+      <c r="C28" s="365" t="inlineStr">
         <is>
           <t>Resolve Pricing API (see backlog)</t>
         </is>
       </c>
-      <c r="D28" s="275" t="inlineStr">
+      <c r="D28" s="366" t="inlineStr">
         <is>
           <t>The macistry.com HAFAS proxy returns no ticket prices. Without accurate pricing, the cost autofill gives wrong break-even calculations for many routes.</t>
         </is>
       </c>
-      <c r="E28" s="394" t="inlineStr">
+      <c r="E28" s="366" t="inlineStr">
         <is>
           <t>🟠 High</t>
         </is>
       </c>
-      <c r="F28" s="275" t="inlineStr">
+      <c r="F28" s="366" t="inlineStr">
         <is>
           <t>M (4-6h)</t>
         </is>
       </c>
-      <c r="G28" s="275" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H28" s="275" t="inlineStr">
-        <is>
-          <t>Pre-launch</t>
-        </is>
-      </c>
-      <c r="I28" s="275" t="inlineStr">
-        <is>
-          <t>Cross-listed from backlog. Elevated to pre-prod because pricing accuracy is the app's core claim.</t>
+      <c r="G28" s="367" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H28" s="368" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="I28" s="369" t="inlineStr">
+        <is>
+          <t>Solved with bundled ÖBB Open Data: fare model fitted to Relationspreise (median deviation 4.9%), editable, remembered per route.</t>
         </is>
       </c>
     </row>
@@ -8145,7 +9222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="238" min="1" max="1"/>
@@ -8167,7 +9244,7 @@
     <row r="2" ht="18" customHeight="1" s="239">
       <c r="A2" s="288" t="inlineStr">
         <is>
-          <t>6 of 7 milestones complete · M7 Production Ready target: 2026-04-12</t>
+          <t>Original plan (Mar 2026): 6 of 7 complete, M7 replaced  ·  Prototype phase (Oct 2026 plan): 4 of 6 complete, M5 next</t>
         </is>
       </c>
     </row>
@@ -8458,7 +9535,7 @@
       </c>
       <c r="D12" s="264" t="inlineStr">
         <is>
-          <t>🔄 In Progress  (30%)</t>
+          <t>⏸ Replaced (Oct 2026 plan)</t>
         </is>
       </c>
       <c r="E12" s="265" t="inlineStr">
@@ -8468,21 +9545,366 @@
       </c>
       <c r="F12" s="265" t="inlineStr">
         <is>
-          <t>Bugs #36/#37 ✓ fixed S13. Remaining: pricing API resolution (PP2), email confirm re-enable (PP1), onboarding rework #44, onboarding images (PP3), App Store assets (PP4), EAS build (PP5)</t>
+          <t>Not finished as planned; continued under the Oct 2026 plan below. Pricing (PP2) solved in S19.</t>
         </is>
       </c>
       <c r="G12" s="265" t="inlineStr">
         <is>
-          <t>S13+</t>
+          <t>S13–S18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="7.5" customHeight="1" s="239">
+      <c r="A13" s="243" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="239">
+      <c r="A14" s="244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PROTOTYPE PHASE — plan of 20 Oct 2026 (details in ROADMAP.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="19.5" customHeight="1" s="239">
+      <c r="A15" s="257" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B15" s="257" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="C15" s="257" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="D15" s="257" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E15" s="257" t="inlineStr">
+        <is>
+          <t>Key Deliverables</t>
+        </is>
+      </c>
+      <c r="F15" s="257" t="inlineStr">
+        <is>
+          <t>Blockers</t>
+        </is>
+      </c>
+      <c r="G15" s="257" t="inlineStr">
+        <is>
+          <t>Sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="51.75" customHeight="1" s="239">
+      <c r="A16" s="421" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="B16" s="421" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C16" s="422" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D16" s="367" t="inlineStr">
+        <is>
+          <t>✅ Complete  (100%)</t>
+        </is>
+      </c>
+      <c r="E16" s="422" t="inlineStr">
+        <is>
+          <t>LF line endings, repo cleanup (Trello/Excel tooling retired), dependencies aligned with SDK 54, dead code and NativeWind removed, one app config, ESLint + Prettier, tsc at 0, Android dev build over USB</t>
+        </is>
+      </c>
+      <c r="F16" s="422" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="422" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="51.75" customHeight="1" s="239">
+      <c r="A17" s="421" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B17" s="421" t="inlineStr">
+        <is>
+          <t>Trip entry + fixes</t>
+        </is>
+      </c>
+      <c r="C17" s="422" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D17" s="367" t="inlineStr">
+        <is>
+          <t>✅ Complete  (100%)</t>
+        </is>
+      </c>
+      <c r="E17" s="422" t="inlineStr">
+        <is>
+          <t>Bundled ÖBB stations (1,117) with autocomplete, rail distance from the GTFS network, fare model (median deviation 4.9%), editable remembered route prices, Check price at ÖBB, anonymous sign-in + optional account, icon/date/crash fixes</t>
+        </is>
+      </c>
+      <c r="F17" s="422" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="422" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="51.75" customHeight="1" s="239">
+      <c r="A18" s="421" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B18" s="421" t="inlineStr">
+        <is>
+          <t>Data core</t>
+        </is>
+      </c>
+      <c r="C18" s="422" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D18" s="367" t="inlineStr">
+        <is>
+          <t>✅ Complete  (100%)</t>
+        </is>
+      </c>
+      <c r="E18" s="422" t="inlineStr">
+        <is>
+          <t>Shared AppData store, XP derived from trips + reward-claim log, app-wide XP feedback, ticket periods + net savings; 76 tests</t>
+        </is>
+      </c>
+      <c r="F18" s="422" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" s="422" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="51.75" customHeight="1" s="239">
+      <c r="A19" s="421" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B19" s="421" t="inlineStr">
+        <is>
+          <t>Cloud backup</t>
+        </is>
+      </c>
+      <c r="C19" s="422" t="inlineStr">
+        <is>
+          <t>2026-11-22 (done 10-21)</t>
+        </is>
+      </c>
+      <c r="D19" s="367" t="inlineStr">
+        <is>
+          <t>✅ Complete  (100%)</t>
+        </is>
+      </c>
+      <c r="E19" s="422" t="inlineStr">
+        <is>
+          <t>Supabase tables with row-level security, local-first background sync, soft deletes, restore on login, merge question for anonymous trips, backup status icon, study export views, −XP toast; 106 tests</t>
+        </is>
+      </c>
+      <c r="F19" s="422" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="422" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="51.75" customHeight="1" s="239">
+      <c r="A20" s="384" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B20" s="384" t="inlineStr">
+        <is>
+          <t>Polish + insights (+ M5b gamification)</t>
+        </is>
+      </c>
+      <c r="C20" s="265" t="inlineStr">
+        <is>
+          <t>2026-12-18</t>
+        </is>
+      </c>
+      <c r="D20" s="264" t="inlineStr">
+        <is>
+          <t>⬜ Next</t>
+        </is>
+      </c>
+      <c r="E20" s="265" t="inlineStr">
+        <is>
+          <t>German + English, edge-to-edge, onboarding rework, insights (saved vs driving, weekly recap, break-even forecast); M5b: weekly goal ladder, fitted quests, journey map, reward revocation</t>
+        </is>
+      </c>
+      <c r="F20" s="265" t="inlineStr">
+        <is>
+          <t>Reminders need expo-notifications (new build)</t>
+        </is>
+      </c>
+      <c r="G20" s="265" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="51.75" customHeight="1" s="239">
+      <c r="A21" s="384" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B21" s="384" t="inlineStr">
+        <is>
+          <t>Study-ready</t>
+        </is>
+      </c>
+      <c r="C21" s="265" t="inlineStr">
+        <is>
+          <t>2027-01-10</t>
+        </is>
+      </c>
+      <c r="D21" s="264" t="inlineStr">
+        <is>
+          <t>⬜ Planned</t>
+        </is>
+      </c>
+      <c r="E21" s="265" t="inlineStr">
+        <is>
+          <t>Privacy notice, study code + consent, own/comparing flag, game switch, 2027 ÖBB data, APK + TestFlight, questionnaires, weekly export</t>
+        </is>
+      </c>
+      <c r="F21" s="265" t="inlineStr">
+        <is>
+          <t>Apple developer account by mid-December; ethics requirement still to ask</t>
+        </is>
+      </c>
+      <c r="G21" s="265" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="51.75" customHeight="1" s="239">
+      <c r="A22" s="384" t="inlineStr">
+        <is>
+          <t>Pilot</t>
+        </is>
+      </c>
+      <c r="B22" s="384" t="inlineStr">
+        <is>
+          <t>Pilot test</t>
+        </is>
+      </c>
+      <c r="C22" s="265" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="D22" s="264" t="inlineStr">
+        <is>
+          <t>⬜ Planned</t>
+        </is>
+      </c>
+      <c r="E22" s="265" t="inlineStr">
+        <is>
+          <t>5–8 people for 2 weeks (30 Nov – 13 Dec), Android only</t>
+        </is>
+      </c>
+      <c r="F22" s="265" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="265" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="51.75" customHeight="1" s="239">
+      <c r="A23" s="384" t="inlineStr">
+        <is>
+          <t>Study</t>
+        </is>
+      </c>
+      <c r="B23" s="384" t="inlineStr">
+        <is>
+          <t>User study</t>
+        </is>
+      </c>
+      <c r="C23" s="265" t="inlineStr">
+        <is>
+          <t>2027-02-21</t>
+        </is>
+      </c>
+      <c r="D23" s="264" t="inlineStr">
+        <is>
+          <t>⬜ Planned</t>
+        </is>
+      </c>
+      <c r="E23" s="265" t="inlineStr">
+        <is>
+          <t>6 weeks (11 Jan – 21 Feb 2027); analysis and writing until submission on 31 Mar 2027</t>
+        </is>
+      </c>
+      <c r="F23" s="265" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G23" s="265" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -8497,7 +9919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="238" min="1" max="1"/>
@@ -8515,7 +9937,7 @@
     <row r="1" ht="43.5" customHeight="1" s="239">
       <c r="A1" s="287" t="inlineStr">
         <is>
-          <t>✅  Complete Feature Registry — 55 Shipped Features</t>
+          <t>✅  Complete Feature Registry — 70 Shipped Features</t>
         </is>
       </c>
     </row>
@@ -11438,6 +12860,756 @@
       <c r="J59" s="443" t="inlineStr">
         <is>
           <t>UX Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1" s="239">
+      <c r="A60" s="438" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="421" t="inlineStr">
+        <is>
+          <t>Trip Export / Import</t>
+        </is>
+      </c>
+      <c r="C60" s="397" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D60" s="439" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="E60" s="440" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="F60" s="369" t="inlineStr">
+        <is>
+          <t>services/tripExport.ts, app/profile.tsx</t>
+        </is>
+      </c>
+      <c r="G60" s="422" t="inlineStr">
+        <is>
+          <t>JSON export via share sheet; import merges by trip ID and skips duplicates; specific error messages added in S19</t>
+        </is>
+      </c>
+      <c r="H60" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I60" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J60" s="443" t="inlineStr">
+        <is>
+          <t>Data Architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1" s="239">
+      <c r="A61" s="438" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="421" t="inlineStr">
+        <is>
+          <t>Anonymous Sign-In</t>
+        </is>
+      </c>
+      <c r="C61" s="397" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D61" s="439" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="E61" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F61" s="369" t="inlineStr">
+        <is>
+          <t>lib/auth.ts, app/index.tsx</t>
+        </is>
+      </c>
+      <c r="G61" s="422" t="inlineStr">
+        <is>
+          <t>Supabase anonymous session on first launch; the app works offline without it</t>
+        </is>
+      </c>
+      <c r="H61" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I61" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J61" s="443" t="inlineStr">
+        <is>
+          <t>Auth Architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="30" customHeight="1" s="239">
+      <c r="A62" s="438" t="n">
+        <v>58</v>
+      </c>
+      <c r="B62" s="421" t="inlineStr">
+        <is>
+          <t>Optional Account Upgrade</t>
+        </is>
+      </c>
+      <c r="C62" s="397" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D62" s="439" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="E62" s="440" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="F62" s="369" t="inlineStr">
+        <is>
+          <t>lib/auth.ts, RegisterForm.tsx</t>
+        </is>
+      </c>
+      <c r="G62" s="422" t="inlineStr">
+        <is>
+          <t>Adds email + password to the same anonymous user ID; logout only for linked accounts</t>
+        </is>
+      </c>
+      <c r="H62" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I62" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J62" s="443" t="inlineStr">
+        <is>
+          <t>Auth Architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="30" customHeight="1" s="239">
+      <c r="A63" s="438" t="n">
+        <v>59</v>
+      </c>
+      <c r="B63" s="421" t="inlineStr">
+        <is>
+          <t>Bundled ÖBB Station Search</t>
+        </is>
+      </c>
+      <c r="C63" s="397" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D63" s="439" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="E63" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F63" s="369" t="inlineStr">
+        <is>
+          <t>services/stations.ts, TripRouteFields.tsx</t>
+        </is>
+      </c>
+      <c r="G63" s="422" t="inlineStr">
+        <is>
+          <t>1,117 stations from ÖBB GTFS with autocomplete; short names on cards</t>
+        </is>
+      </c>
+      <c r="H63" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I63" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J63" s="443" t="inlineStr">
+        <is>
+          <t>Data Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="30" customHeight="1" s="239">
+      <c r="A64" s="438" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="421" t="inlineStr">
+        <is>
+          <t>Rail Distance (GTFS Network)</t>
+        </is>
+      </c>
+      <c r="C64" s="397" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D64" s="439" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="E64" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F64" s="369" t="inlineStr">
+        <is>
+          <t>services/stations.ts, assets/data/network.json</t>
+        </is>
+      </c>
+      <c r="G64" s="422" t="inlineStr">
+        <is>
+          <t>Offline Dijkstra on the GTFS track network; straight-line fallback</t>
+        </is>
+      </c>
+      <c r="H64" s="441" t="inlineStr">
+        <is>
+          <t>Affects XP</t>
+        </is>
+      </c>
+      <c r="I64" s="442" t="inlineStr">
+        <is>
+          <t>Distance as effort proxy; Eco-feedback systems (Froehlich et al. 2010)</t>
+        </is>
+      </c>
+      <c r="J64" s="443" t="inlineStr">
+        <is>
+          <t>Data Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="30" customHeight="1" s="239">
+      <c r="A65" s="438" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="421" t="inlineStr">
+        <is>
+          <t>Fare Estimate Model</t>
+        </is>
+      </c>
+      <c r="C65" s="397" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D65" s="439" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="E65" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F65" s="369" t="inlineStr">
+        <is>
+          <t>services/fareEstimate.ts, scripts/data/</t>
+        </is>
+      </c>
+      <c r="G65" s="422" t="inlineStr">
+        <is>
+          <t>Price from distance fitted to ÖBB Relationspreise (median deviation 4.9%); editable, remembered per route; Verbund hint</t>
+        </is>
+      </c>
+      <c r="H65" s="441" t="inlineStr">
+        <is>
+          <t>Affects savings</t>
+        </is>
+      </c>
+      <c r="I65" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J65" s="443" t="inlineStr">
+        <is>
+          <t>Data Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="30" customHeight="1" s="239">
+      <c r="A66" s="438" t="n">
+        <v>62</v>
+      </c>
+      <c r="B66" s="421" t="inlineStr">
+        <is>
+          <t>Check Price at ÖBB</t>
+        </is>
+      </c>
+      <c r="C66" s="397" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="D66" s="439" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="E66" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F66" s="369" t="inlineStr">
+        <is>
+          <t>services/oebbLinks.ts, CheckPriceLink.tsx</t>
+        </is>
+      </c>
+      <c r="G66" s="422" t="inlineStr">
+        <is>
+          <t>Opens the ÖBB timetable with the route pre-filled</t>
+        </is>
+      </c>
+      <c r="H66" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I66" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J66" s="443" t="inlineStr">
+        <is>
+          <t>UX Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="30" customHeight="1" s="239">
+      <c r="A67" s="438" t="n">
+        <v>63</v>
+      </c>
+      <c r="B67" s="421" t="inlineStr">
+        <is>
+          <t>Shared AppData Store</t>
+        </is>
+      </c>
+      <c r="C67" s="397" t="inlineStr">
+        <is>
+          <t>Refactor</t>
+        </is>
+      </c>
+      <c r="D67" s="439" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="E67" s="440" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="F67" s="369" t="inlineStr">
+        <is>
+          <t>store/AppData.tsx</t>
+        </is>
+      </c>
+      <c r="G67" s="422" t="inlineStr">
+        <is>
+          <t>One store for trips, reward claims and the profile; screens never touch storage</t>
+        </is>
+      </c>
+      <c r="H67" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I67" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J67" s="443" t="inlineStr">
+        <is>
+          <t>Software Quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="30" customHeight="1" s="239">
+      <c r="A68" s="438" t="n">
+        <v>64</v>
+      </c>
+      <c r="B68" s="421" t="inlineStr">
+        <is>
+          <t>Derived XP + Reward Claim Log</t>
+        </is>
+      </c>
+      <c r="C68" s="397" t="inlineStr">
+        <is>
+          <t>Gamification</t>
+        </is>
+      </c>
+      <c r="D68" s="439" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="E68" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F68" s="369" t="inlineStr">
+        <is>
+          <t>utils/rewards.ts, store/AppData.tsx</t>
+        </is>
+      </c>
+      <c r="G68" s="422" t="inlineStr">
+        <is>
+          <t>XP = trip XP + claimed rewards with timestamps; one-time migration of the old layout</t>
+        </is>
+      </c>
+      <c r="H68" s="441" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="I68" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J68" s="443" t="inlineStr">
+        <is>
+          <t>Gamification Design / Research Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="30" customHeight="1" s="239">
+      <c r="A69" s="438" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="421" t="inlineStr">
+        <is>
+          <t>Ticket Periods + Net Savings</t>
+        </is>
+      </c>
+      <c r="C69" s="397" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D69" s="439" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="E69" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F69" s="369" t="inlineStr">
+        <is>
+          <t>utils/ticketPeriod.ts, FinancialOverview.tsx</t>
+        </is>
+      </c>
+      <c r="G69" s="422" t="inlineStr">
+        <is>
+          <t>Break-even per ticket year from the start date; net savings after break-even</t>
+        </is>
+      </c>
+      <c r="H69" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I69" s="442" t="inlineStr">
+        <is>
+          <t>Goal-setting theory (Locke &amp; Latham 1990)</t>
+        </is>
+      </c>
+      <c r="J69" s="443" t="inlineStr">
+        <is>
+          <t>Feature Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1" s="239">
+      <c r="A70" s="438" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="421" t="inlineStr">
+        <is>
+          <t>Cloud Backup (Supabase)</t>
+        </is>
+      </c>
+      <c r="C70" s="397" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D70" s="439" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="E70" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F70" s="369" t="inlineStr">
+        <is>
+          <t>supabase/migrations/, utils/syncLogic.ts, services/cloudSync.ts, store/AppData.tsx</t>
+        </is>
+      </c>
+      <c r="G70" s="422" t="inlineStr">
+        <is>
+          <t>Local-first sync of trips, rewards and profile with row-level security; offline queue, soft deletes, restore on login</t>
+        </is>
+      </c>
+      <c r="H70" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I70" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J70" s="443" t="inlineStr">
+        <is>
+          <t>Data Architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1" s="239">
+      <c r="A71" s="438" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="421" t="inlineStr">
+        <is>
+          <t>Merge Question on Login</t>
+        </is>
+      </c>
+      <c r="C71" s="397" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D71" s="439" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="E71" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F71" s="369" t="inlineStr">
+        <is>
+          <t>AccountMergePrompt.tsx, store/AppData.tsx</t>
+        </is>
+      </c>
+      <c r="G71" s="422" t="inlineStr">
+        <is>
+          <t>"Add the N trips from this phone to your account?" Yes merges, No keeps the account's data</t>
+        </is>
+      </c>
+      <c r="H71" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J71" s="443" t="inlineStr">
+        <is>
+          <t>Auth Architecture / Privacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1" s="239">
+      <c r="A72" s="438" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="421" t="inlineStr">
+        <is>
+          <t>Backup Status Icon</t>
+        </is>
+      </c>
+      <c r="C72" s="397" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="D72" s="439" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="E72" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F72" s="369" t="inlineStr">
+        <is>
+          <t>SyncStatusBadge.tsx</t>
+        </is>
+      </c>
+      <c r="G72" s="422" t="inlineStr">
+        <is>
+          <t>Red cloud on the main screen only while the backup fails; tap for details and retry</t>
+        </is>
+      </c>
+      <c r="H72" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" s="442" t="inlineStr">
+        <is>
+          <t>Visibility of system status (Nielsen 1994)</t>
+        </is>
+      </c>
+      <c r="J72" s="443" t="inlineStr">
+        <is>
+          <t>UX Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1" s="239">
+      <c r="A73" s="438" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" s="421" t="inlineStr">
+        <is>
+          <t>Study Export Views</t>
+        </is>
+      </c>
+      <c r="C73" s="397" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D73" s="439" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="E73" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F73" s="369" t="inlineStr">
+        <is>
+          <t>supabase/migrations/ (schema study)</t>
+        </is>
+      </c>
+      <c r="G73" s="422" t="inlineStr">
+        <is>
+          <t>Trips, rewards and tickets without station names; merged anonymous users left out</t>
+        </is>
+      </c>
+      <c r="H73" s="471" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="442" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J73" s="443" t="inlineStr">
+        <is>
+          <t>Research Data / Privacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="30" customHeight="1" s="239">
+      <c r="A74" s="438" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="421" t="inlineStr">
+        <is>
+          <t>−XP Toast</t>
+        </is>
+      </c>
+      <c r="C74" s="397" t="inlineStr">
+        <is>
+          <t>Gamification</t>
+        </is>
+      </c>
+      <c r="D74" s="439" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="E74" s="440" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F74" s="369" t="inlineStr">
+        <is>
+          <t>XPToast.tsx, RewardFeedback.tsx</t>
+        </is>
+      </c>
+      <c r="G74" s="422" t="inlineStr">
+        <is>
+          <t>Red toast that sinks when deleting or editing a trip lowers XP</t>
+        </is>
+      </c>
+      <c r="H74" s="441" t="inlineStr">
+        <is>
+          <t>Delete: −XP</t>
+        </is>
+      </c>
+      <c r="I74" s="442" t="inlineStr">
+        <is>
+          <t>Immediate feedback principle (Hattie &amp; Timperley 2007)</t>
+        </is>
+      </c>
+      <c r="J74" s="443" t="inlineStr">
+        <is>
+          <t>Gamification Theory</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roadmap: add trip search/filter, CO₂ source, final test round; close stale backlog items
From the PM spreadsheet's open backlog: #46 search/filter and a citable
CO₂ factor go to M5, the final Android + iPhone test round (PP5) to M6.
Spreadsheet: route prices, #50 and PP3 marked done (no longer needed or
already there); dashboard counts adjusted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KlimaChallenge_PM_v5.xlsx
+++ b/docs/KlimaChallenge_PM_v5.xlsx
@@ -2412,7 +2412,7 @@
       <c r="D6" s="251" t="n"/>
       <c r="E6" s="253" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F6" s="251" t="n"/>
@@ -2424,7 +2424,7 @@
       <c r="H6" s="251" t="n"/>
       <c r="I6" s="255" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J6" s="251" t="n"/>
@@ -6610,49 +6610,49 @@
       </c>
     </row>
     <row r="12" ht="48" customHeight="1" s="239">
-      <c r="A12" s="372" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B12" s="372" t="inlineStr">
+      <c r="A12" s="365" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B12" s="366" t="inlineStr">
         <is>
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="C12" s="372" t="inlineStr">
+      <c r="C12" s="365" t="inlineStr">
         <is>
           <t>More prefetched route prices</t>
         </is>
       </c>
-      <c r="D12" s="372" t="inlineStr">
+      <c r="D12" s="366" t="inlineStr">
         <is>
           <t>Add Graz, Salzburg, Innsbruck, Linz routes to ROUTE_PRICES in TripRouteFields.tsx. Currently only Villach routes.</t>
         </is>
       </c>
-      <c r="E12" s="373" t="inlineStr">
+      <c r="E12" s="366" t="inlineStr">
         <is>
           <t>🔵 Low</t>
         </is>
       </c>
-      <c r="F12" s="372" t="inlineStr">
+      <c r="F12" s="366" t="inlineStr">
         <is>
           <t>XS (1h)</t>
         </is>
       </c>
-      <c r="G12" s="372" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H12" s="372" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="I12" s="372" t="inlineStr">
-        <is>
-          <t>Quick win for Austria-wide usability pending proper pricing API</t>
+      <c r="G12" s="367" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H12" s="368" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="I12" s="369" t="inlineStr">
+        <is>
+          <t>No longer needed: the ÖBB fare model (S19) estimates prices for all of Austria.</t>
         </is>
       </c>
     </row>
@@ -6935,7 +6935,7 @@
       </c>
       <c r="I19" s="386" t="inlineStr">
         <is>
-          <t>Filter bar above trip list in user.tsx. Client-side filtering on trips array — no API needed.</t>
+          <t>Filter bar above trip list in user.tsx. Client-side filtering on trips array — no API needed. → Now in ROADMAP.md (M5).</t>
         </is>
       </c>
     </row>
@@ -7081,49 +7081,49 @@
       </c>
     </row>
     <row r="23" ht="48" customHeight="1" s="239">
-      <c r="A23" s="389" t="inlineStr">
+      <c r="A23" s="365" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="B23" s="331" t="inlineStr">
+      <c r="B23" s="366" t="inlineStr">
         <is>
           <t>Tech Debt</t>
         </is>
       </c>
-      <c r="C23" s="389" t="inlineStr">
+      <c r="C23" s="365" t="inlineStr">
         <is>
           <t>Clean up stale XP seeding comment in user.tsx</t>
         </is>
       </c>
-      <c r="D23" s="331" t="inlineStr">
+      <c r="D23" s="366" t="inlineStr">
         <is>
           <t>Comment references ensuring 10 hardcoded dummy trips grant XP on fresh installs — no longer true after #37 fix.</t>
         </is>
       </c>
-      <c r="E23" s="390" t="inlineStr">
+      <c r="E23" s="366" t="inlineStr">
         <is>
           <t>🔵 Low</t>
         </is>
       </c>
-      <c r="F23" s="331" t="inlineStr">
+      <c r="F23" s="366" t="inlineStr">
         <is>
           <t>XS (5m)</t>
         </is>
       </c>
-      <c r="G23" s="331" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H23" s="331" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="I23" s="332" t="inlineStr">
-        <is>
-          <t>One-line comment update in the XP init useEffect block in user.tsx.</t>
+      <c r="G23" s="367" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H23" s="368" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="I23" s="369" t="inlineStr">
+        <is>
+          <t>No longer needed: the XP seeding code was removed when XP became derived from trips (M3).</t>
         </is>
       </c>
     </row>
@@ -7323,49 +7323,49 @@
       </c>
     </row>
     <row r="29" ht="25.5" customHeight="1" s="239">
-      <c r="A29" s="265" t="inlineStr">
+      <c r="A29" s="365" t="inlineStr">
         <is>
           <t>PP3</t>
         </is>
       </c>
-      <c r="B29" s="265" t="inlineStr">
+      <c r="B29" s="366" t="inlineStr">
         <is>
           <t>Pre-Prod</t>
         </is>
       </c>
-      <c r="C29" s="265" t="inlineStr">
+      <c r="C29" s="365" t="inlineStr">
         <is>
           <t>Add onboarding images</t>
         </is>
       </c>
-      <c r="D29" s="265" t="inlineStr">
+      <c r="D29" s="366" t="inlineStr">
         <is>
           <t>onboard1.png, onboard2.png, loginbg.png missing from assets/images/. Metro bundler fails without them — app cannot be built.</t>
         </is>
       </c>
-      <c r="E29" s="385" t="inlineStr">
+      <c r="E29" s="366" t="inlineStr">
         <is>
           <t>🟡 Medium</t>
         </is>
       </c>
-      <c r="F29" s="265" t="inlineStr">
+      <c r="F29" s="366" t="inlineStr">
         <is>
           <t>S (design)</t>
         </is>
       </c>
-      <c r="G29" s="265" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H29" s="265" t="inlineStr">
-        <is>
-          <t>Pre-launch</t>
-        </is>
-      </c>
-      <c r="I29" s="265" t="inlineStr">
-        <is>
-          <t>Slide 1: ROI annotated map. Slide 2: full KlimaTicket coverage map. loginbg: plain Austrian map.</t>
+      <c r="G29" s="367" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H29" s="368" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I29" s="369" t="inlineStr">
+        <is>
+          <t>Done: onboard1.png, onboard2.png and loginbg.png are in assets/images.</t>
         </is>
       </c>
     </row>
@@ -7459,7 +7459,7 @@
       </c>
       <c r="I31" s="265" t="inlineStr">
         <is>
-          <t>Test on physical devices not just simulator. Verify Supabase session persistence across app restarts.</t>
+          <t>Test on physical devices not just simulator. Verify Supabase session persistence across app restarts. → Now in ROADMAP.md (M6).</t>
         </is>
       </c>
     </row>

</xml_diff>